<commit_message>
feat: redesign export Excel bergaya laporan korporat (header perusahaan, band kelompok kolom, footer resmi)
</commit_message>
<xml_diff>
--- a/examples/laporan_reasuransi_contoh.xlsx
+++ b/examples/laporan_reasuransi_contoh.xlsx
@@ -12,17 +12,18 @@
     <sheet name="Ringkasan Keuangan" sheetId="3" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Borderaux Premi'!$A$3:$H$6</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Borderaux Premi'!$3:$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Borderaux Klaim'!$A$3:$J$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Borderaux Klaim'!$3:$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Borderaux Premi'!$A$6:$H$9</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Borderaux Premi'!$1:$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Borderaux Klaim'!$A$6:$J$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Borderaux Klaim'!$1:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Ringkasan Keuangan'!$1:$6</definedName>
   </definedNames>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="61">
   <si>
     <t>No Polis</t>
   </si>
@@ -78,7 +79,34 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>Laporan Produksi &amp; Premi Reasuransi (Borderaux Premi)</t>
+    <t>DESWA INVISCO MULTITAMA</t>
+  </si>
+  <si>
+    <t>LAPORAN PRODUKSI &amp; PREMI REASURANSI — BORDERAUX PREMI</t>
+  </si>
+  <si>
+    <t>No. Dok : RR-2026-09    |    Periode : September 2026    |    Tanggal Cetak : 16/09/2026 14:43</t>
+  </si>
+  <si>
+    <t>INFORMASI POLIS</t>
+  </si>
+  <si>
+    <t>UANG PERTANGGUNGAN (Rp)</t>
+  </si>
+  <si>
+    <t>REASURANSI</t>
+  </si>
+  <si>
+    <t>Dibuat oleh,</t>
+  </si>
+  <si>
+    <t>Disetujui oleh,</t>
+  </si>
+  <si>
+    <t>( Nama &amp; Tanda Tangan )</t>
+  </si>
+  <si>
+    <t>Dokumen ini dibuat otomatis oleh Sistem Laporan Reasuransi pada 16/09/2026 14:43. Data disajikan sesuai input yang tercatat di sistem.</t>
   </si>
   <si>
     <t>No Klaim</t>
@@ -114,7 +142,19 @@
     <t>Under Investigation</t>
   </si>
   <si>
-    <t>Laporan Klaim Reasuransi (Borderaux Klaim)</t>
+    <t>LAPORAN KLAIM REASURANSI — BORDERAUX KLAIM</t>
+  </si>
+  <si>
+    <t>KODE</t>
+  </si>
+  <si>
+    <t>DATA TERTANGGUNG</t>
+  </si>
+  <si>
+    <t>NILAI KLAIM (Rp)</t>
+  </si>
+  <si>
+    <t>STATUS</t>
   </si>
   <si>
     <t>Metrik</t>
@@ -162,7 +202,10 @@
     <t>Premi netto dikurangi recovery klaim</t>
   </si>
   <si>
-    <t>Ringkasan Akun Keuangan Reasuransi</t>
+    <t>RINGKASAN AKUN KEUANGAN REASURANSI</t>
+  </si>
+  <si>
+    <t>RINGKASAN AKUN KEUANGAN</t>
   </si>
 </sst>
 </file>
@@ -173,7 +216,7 @@
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="11">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -188,7 +231,34 @@
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
-      <sz val="14"/>
+      <sz val="16"/>
+      <color rgb="FF1F3864"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="13"/>
+      <color rgb="FF1F3864"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="9"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="9"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
@@ -197,7 +267,7 @@
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
-      <sz val="11"/>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
@@ -206,17 +276,65 @@
       <i val="0"/>
       <strike val="0"/>
       <u val="none"/>
-      <sz val="11"/>
+      <sz val="10.5"/>
+      <color rgb="FF1F3864"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="8"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="1"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="8"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="10.5"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -226,24 +344,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2E74B5"/>
+        <fgColor rgb="FFF2F7FC"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9E1F2"/>
+        <fgColor rgb="FFBDD7EE"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -253,16 +365,136 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFA6A6A6"/>
+        <color rgb="FFC8CDD2"/>
       </left>
       <right style="thin">
-        <color rgb="FFA6A6A6"/>
+        <color rgb="FFC8CDD2"/>
       </right>
       <top style="thin">
-        <color rgb="FFA6A6A6"/>
+        <color rgb="FFC8CDD2"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFA6A6A6"/>
+        <color rgb="FFC8CDD2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F3864"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFC8CDD2"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1F3864"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFC8CDD2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC8CDD2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFC8CDD2"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1F3864"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFC8CDD2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC8CDD2"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F3864"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1F3864"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFC8CDD2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F3864"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFC8CDD2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFC8CDD2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFC8CDD2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC8CDD2"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F3864"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFC8CDD2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFC8CDD2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC8CDD2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFC8CDD2"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF2E74B5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F3864"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC8CDD2"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1F3864"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF2E74B5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F3864"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1F3864"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFC8CDD2"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF2E74B5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1F3864"/>
       </bottom>
       <diagonal/>
     </border>
@@ -270,83 +502,124 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="42">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="3" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="4" numFmtId="0" fillId="3" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="4" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="4" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="4" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="4" borderId="3" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="5" numFmtId="0" fillId="4" borderId="4" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="5" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="5" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="5" borderId="5" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="164" fillId="0" borderId="1" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="164" fillId="5" borderId="1" applyFont="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="164" fillId="4" borderId="1" applyFont="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="5" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="164" fillId="0" borderId="1" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="3" fillId="4" borderId="1" applyFont="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="3" fillId="0" borderId="1" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="4" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="0" numFmtId="3" fillId="5" borderId="1" applyFont="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="5" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="3" numFmtId="3" fillId="5" borderId="1" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="4" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="5" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="3" fillId="0" borderId="6" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="3" fillId="5" borderId="6" applyFont="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="4" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="5" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="6" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="6" borderId="8" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="3" fillId="6" borderId="8" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="6" borderId="9" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="6" numFmtId="0" fillId="6" borderId="7" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="7" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="8" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="9" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="6" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="5" borderId="6" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="4" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="6" numFmtId="3" fillId="6" borderId="7" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="5" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="5" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="3" fillId="4" borderId="1" applyFont="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="0" numFmtId="3" fillId="0" borderId="1" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
     <xf xfId="0" fontId="0" numFmtId="165" fillId="0" borderId="1" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="0" numFmtId="3" fillId="0" borderId="1" applyFont="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="6" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="10" numFmtId="0" fillId="3" borderId="9" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="10" numFmtId="3" fillId="3" borderId="7" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="3" numFmtId="3" fillId="5" borderId="1" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="4" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="1" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="5" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    <xf xfId="0" fontId="10" numFmtId="0" fillId="3" borderId="8" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -648,7 +921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="true" style="0"/>
@@ -661,145 +934,221 @@
     <col min="8" max="8" width="22" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" customHeight="1" ht="28">
+    <row r="1" spans="1:8" customHeight="1" ht="32">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="3" spans="1:8" customHeight="1" ht="32">
+    </row>
+    <row r="2" spans="1:8" customHeight="1" ht="7"/>
+    <row r="3" spans="1:8" customHeight="1" ht="28">
       <c r="A3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" customHeight="1" ht="18">
+      <c r="A4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5" spans="1:8" customHeight="1" ht="22">
+      <c r="A5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" s="4"/>
+    </row>
+    <row r="6" spans="1:8" customHeight="1" ht="34">
+      <c r="A6" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B6" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C6" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D6" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E6" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H6" s="8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="5" t="s">
+    <row r="7" spans="1:8">
+      <c r="A7" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B7" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C7" s="12">
         <v>31118.0</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D7" s="16">
         <v>1000000000.0</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E7" s="16">
         <v>400000000.0</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F7" s="16">
         <v>600000000.0</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G7" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="9">
+      <c r="H7" s="20">
         <v>30000000.0</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="6" t="s">
+    <row r="8" spans="1:8">
+      <c r="A8" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B8" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C8" s="13">
         <v>33079.0</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D8" s="17">
         <v>500000000.0</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E8" s="17">
         <v>100000000.0</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F8" s="17">
         <v>400000000.0</v>
       </c>
-      <c r="G5" s="12" t="s">
+      <c r="G8" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H8" s="21">
         <v>15000000.0</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="5" t="s">
+    <row r="9" spans="1:8">
+      <c r="A9" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B9" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C9" s="12">
         <v>28796.0</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D9" s="16">
         <v>750000000.0</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E9" s="16">
         <v>350000000.0</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F9" s="16">
         <v>400000000.0</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G9" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="9">
+      <c r="H9" s="20">
         <v>15000000.0</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="13" t="s">
+    <row r="10" spans="1:8">
+      <c r="A10" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="14">
-        <f>SUM(H4:H6)</f>
-      </c>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="26">
+        <f>SUM(H7:H9)</f>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="29" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" customHeight="1" ht="34"/>
+    <row r="14" spans="1:8">
+      <c r="A14" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" s="30" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="31"/>
+      <c r="C16" s="31"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H6"/>
+  <autoFilter ref="A6:H9"/>
   <mergeCells>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="E12:H12"/>
+    <mergeCell ref="A14:D14"/>
+    <mergeCell ref="E14:H14"/>
+    <mergeCell ref="A16:H16"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.7" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="landscape" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddFooter>&amp;LDESWA INVISCO MULTITAMA&amp;CHalaman &amp;P dari &amp;N&amp;RDicetak: &amp;D &amp;T</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -809,7 +1158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="true" style="0"/>
@@ -824,143 +1173,228 @@
     <col min="10" max="10" width="20" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" customHeight="1" ht="28">
+    <row r="1" spans="1:10" customHeight="1" ht="32">
       <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" customHeight="1" ht="7"/>
+    <row r="3" spans="1:10" customHeight="1" ht="28">
+      <c r="A3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" spans="1:10" customHeight="1" ht="18">
+      <c r="A4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+    </row>
+    <row r="5" spans="1:10" customHeight="1" ht="22">
+      <c r="A5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" customHeight="1" ht="34">
+      <c r="A6" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-    </row>
-    <row r="3" spans="1:10" customHeight="1" ht="32">
-      <c r="A3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="2" t="s">
+      <c r="G6" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I3" s="2" t="s">
+      <c r="H6" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="I6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
-      <c r="A4" s="5" t="s">
+      <c r="J6" s="8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="12">
+        <v>31118.0</v>
+      </c>
+      <c r="F7" s="16">
+        <v>100000000.0</v>
+      </c>
+      <c r="G7" s="16">
+        <v>1000000000.0</v>
+      </c>
+      <c r="H7" s="16">
+        <v>20000000.0</v>
+      </c>
+      <c r="I7" s="16">
+        <v>600000000.0</v>
+      </c>
+      <c r="J7" s="32" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="13">
+        <v>33079.0</v>
+      </c>
+      <c r="F8" s="17">
+        <v>80000000.0</v>
+      </c>
+      <c r="G8" s="17">
+        <v>500000000.0</v>
+      </c>
+      <c r="H8" s="17">
+        <v>15000000.0</v>
+      </c>
+      <c r="I8" s="17">
+        <v>400000000.0</v>
+      </c>
+      <c r="J8" s="33" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="34">
+        <f>SUM(F7:F8)</f>
+      </c>
+      <c r="G9" s="24"/>
+      <c r="H9" s="34">
+        <f>SUM(H7:H8)</f>
+      </c>
+      <c r="I9" s="24"/>
+      <c r="J9" s="25"/>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="15" t="s">
+      <c r="F11" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="7">
-        <v>31118.0</v>
-      </c>
-      <c r="F4" s="9">
-        <v>100000000.0</v>
-      </c>
-      <c r="G4" s="9">
-        <v>1000000000.0</v>
-      </c>
-      <c r="H4" s="9">
-        <v>20000000.0</v>
-      </c>
-      <c r="I4" s="9">
-        <v>600000000.0</v>
-      </c>
-      <c r="J4" s="17" t="s">
+    </row>
+    <row r="12" spans="1:10" customHeight="1" ht="34"/>
+    <row r="13" spans="1:10">
+      <c r="A13" s="30" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="5" spans="1:10">
-      <c r="A5" s="6" t="s">
+      <c r="F13" s="30" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="A15" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="E5" s="8">
-        <v>33079.0</v>
-      </c>
-      <c r="F5" s="10">
-        <v>80000000.0</v>
-      </c>
-      <c r="G5" s="10">
-        <v>500000000.0</v>
-      </c>
-      <c r="H5" s="10">
-        <v>15000000.0</v>
-      </c>
-      <c r="I5" s="10">
-        <v>400000000.0</v>
-      </c>
-      <c r="J5" s="18" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="14">
-        <f>SUM(F4:F5)</f>
-      </c>
-      <c r="G6" s="13"/>
-      <c r="H6" s="14">
-        <f>SUM(H4:H5)</f>
-      </c>
-      <c r="I6" s="13"/>
-      <c r="J6" s="13"/>
+      <c r="B15" s="31"/>
+      <c r="C15" s="31"/>
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="31"/>
+      <c r="H15" s="31"/>
+      <c r="I15" s="31"/>
+      <c r="J15" s="31"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J5"/>
+  <autoFilter ref="A6:J8"/>
   <mergeCells>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="J5:J5"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="F11:J11"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="F13:J13"/>
+    <mergeCell ref="A15:J15"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.7" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="landscape" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddFooter>&amp;LDESWA INVISCO MULTITAMA&amp;CHalaman &amp;P dari &amp;N&amp;RDicetak: &amp;D &amp;T</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -968,105 +1402,161 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="true" style="0"/>
     <col min="2" max="2" width="24" customWidth="true" style="0"/>
-    <col min="3" max="3" width="46" customWidth="true" style="0"/>
+    <col min="3" max="3" width="52" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" customHeight="1" ht="28">
+    <row r="1" spans="1:3" customHeight="1" ht="32">
       <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" customHeight="1" ht="7"/>
+    <row r="3" spans="1:3" customHeight="1" ht="28">
+      <c r="A3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" customHeight="1" ht="18">
+      <c r="A4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5" spans="1:3" customHeight="1" ht="22">
+      <c r="A5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+    </row>
+    <row r="6" spans="1:3" customHeight="1" ht="34">
+      <c r="A6" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="3" spans="1:3" customHeight="1" ht="32">
-      <c r="A3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" s="22">
-        <f>SUM('Borderaux Premi'!H4:H6)</f>
-      </c>
-      <c r="C4" s="26" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="23">
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="35" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="36">
+        <f>SUM('Borderaux Premi'!H7:H9)</f>
+      </c>
+      <c r="C7" s="38" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="37">
         <v>0.1</v>
       </c>
-      <c r="C5" s="27" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="22">
-        <f>B4*B5</f>
-      </c>
-      <c r="C6" s="26" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="24">
-        <f>B4-B6</f>
-      </c>
-      <c r="C7" s="27" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="B8" s="22">
-        <f>SUM('Borderaux Klaim'!H4:H5)</f>
-      </c>
-      <c r="C8" s="26" t="s">
-        <v>43</v>
+      <c r="C8" s="38" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" s="21" t="s">
-        <v>44</v>
-      </c>
-      <c r="B9" s="25">
-        <f>B7-B8</f>
-      </c>
-      <c r="C9" s="28" t="s">
-        <v>45</v>
-      </c>
+      <c r="A9" s="35" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="36">
+        <f>B7*B8</f>
+      </c>
+      <c r="C9" s="38" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" s="36">
+        <f>B7-B9</f>
+      </c>
+      <c r="C10" s="38" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="35" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" s="36">
+        <f>SUM('Borderaux Klaim'!H7:H8)</f>
+      </c>
+      <c r="C11" s="38" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="39" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="40">
+        <f>B10-B11</f>
+      </c>
+      <c r="C12" s="41" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="29" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" customHeight="1" ht="34"/>
+    <row r="16" spans="1:3">
+      <c r="A16" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="30" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
     </row>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A14:A14"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="A16:A16"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="A18:C18"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.7" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="landscape" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddFooter>&amp;LDESWA INVISCO MULTITAMA&amp;CHalaman &amp;P dari &amp;N&amp;RDicetak: &amp;D &amp;T</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>